<commit_message>
Refresh temporary review from current local build
</commit_message>
<xml_diff>
--- a/review/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
+++ b/review/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R65e26a26fe2d41c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="Reff7820588f04295"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R2867df89e0684d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R841b0fada9274cd0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,7 +2313,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra255213e202344c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f24b876eb14d32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2841,7 +2841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfea9a80a95fe489e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R204719ebd797405d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>